<commit_message>
chore: crawl 2026-09-08 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G215"/>
+  <dimension ref="A1:G216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3674,24 +3674,20 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 87kb</t>
+          <t>Edital n° 26/2026 - Programas CAPES/MATH/STIC/CLIMAT-AMSUD, formato - pdf, 237kb</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/26022024_Edital_2328837_SEI_2326326_Edital_02_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2891614_sei_2891436_edital_26_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2</v>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16052024_Edital_2379426_SEI_2379169_Edital_02_2024.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3701,20 +3697,24 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
+          <t>Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 87kb</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/26022024_Edital_2328837_SEI_2326326_Edital_02_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>1</v>
-      </c>
-      <c r="G114" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16052024_Edital_2379426_SEI_2379169_Edital_02_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3724,24 +3724,20 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>3</v>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3751,22 +3747,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
+          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3778,22 +3774,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3805,22 +3801,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
+          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3832,22 +3828,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
+          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3859,22 +3855,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
+          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3886,22 +3882,22 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
+          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3913,20 +3909,24 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>1</v>
-      </c>
-      <c r="G122" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3936,14 +3936,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Edital nº 14/2025 - PCI - pdf, 83kb</t>
+          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31072025_Edital_2646654_SEI_2644987_Edital_14_2025.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -3959,24 +3959,20 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
+          <t>Edital nº 14/2025 - PCI - pdf, 83kb</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31072025_Edital_2646654_SEI_2644987_Edital_14_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2</v>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3986,20 +3982,24 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
+          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>1</v>
-      </c>
-      <c r="G125" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4009,14 +4009,14 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
+          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -4032,14 +4032,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
+          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -4055,24 +4055,20 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
+          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>3</v>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4082,14 +4078,14 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 281kb</t>
+          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24082023_Edital_2043434_Edital_21_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -4097,7 +4093,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Retificação do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/01112023_Edital_2262651_SEI_2262236_Edital_21_2023.pdf/@@display-file/file ; Alteração do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31102023_Edital_2261925_SEI_2261451_Edital_22_2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4109,20 +4105,24 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
+          <t>Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 281kb</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24082023_Edital_2043434_Edital_21_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
-      </c>
-      <c r="G130" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/01112023_Edital_2262651_SEI_2262236_Edital_21_2023.pdf/@@display-file/file ; Alteração do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31102023_Edital_2261925_SEI_2261451_Edital_22_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4132,24 +4132,20 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
+          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4159,22 +4155,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
+          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F132" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file ; Relação dos Programas de Pós-Graduação (PPGs) - Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 1.836kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/resultado_2881142_pdai_divulgacao_ppgs_bolsas_v-final_13-08-2026.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4186,22 +4182,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
+          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file ; Relação dos Programas de Pós-Graduação (PPGs) - Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 1.836kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/resultado_2881142_pdai_divulgacao_ppgs_bolsas_v-final_13-08-2026.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4213,20 +4209,24 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Edital nº 24/2026 - Cooperação entre Instituições para</t>
+          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878169_edital_24_2026___pci.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1</v>
-      </c>
-      <c r="G134" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4236,24 +4236,20 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
+          <t>Edital nº 24/2026 - Cooperação entre Instituições para</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878169_edital_24_2026___pci.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>3</v>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4263,22 +4259,22 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 83kb</t>
+          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/17092024_Edital_2461148_SEI_2460992_Edital_25_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10122024_Edital_2510251_SEI_2508924_Edital_25_2024___Alteracao.pdf/@@display-file/file</t>
+          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4290,20 +4286,24 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Edital nº 25/2026 - Edição 2027, formato, pdf, 145kb</t>
+          <t>Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 83kb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2886643_sei_2886062_edital_n___25_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/17092024_Edital_2461148_SEI_2460992_Edital_25_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>1</v>
-      </c>
-      <c r="G137" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10122024_Edital_2510251_SEI_2508924_Edital_25_2024___Alteracao.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4313,24 +4313,20 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
+          <t>Edital nº 25/2026 - Edição 2027, formato, pdf, 145kb</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2886643_sei_2886062_edital_n___25_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>3</v>
-      </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4340,22 +4336,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
+          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4367,22 +4363,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
+          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
+          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4394,14 +4390,14 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
+          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -4409,7 +4405,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
+          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4421,14 +4417,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
+          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -4436,7 +4432,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4448,22 +4444,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
+          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4475,20 +4471,24 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
+          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F144" t="n">
-        <v>1</v>
-      </c>
-      <c r="G144" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4498,14 +4498,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
+          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -4521,24 +4521,20 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
+          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F146" t="n">
-        <v>3</v>
-      </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4548,22 +4544,22 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4575,20 +4571,24 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
+          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F148" t="n">
-        <v>1</v>
-      </c>
-      <c r="G148" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4598,24 +4598,20 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
+          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F149" t="n">
-        <v>2</v>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4625,22 +4621,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 06/2022 - formato, pdf, 331kb</t>
+          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02022022_Edital_1626836_SEI_CAPES___1626182___Edita_6.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
         </is>
       </c>
       <c r="F150" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Alteração do Edital PAEP nº 06/2022 - formato, pdf, 80kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15062022_Edital_1733665_Edital_6_2022.pdf/@@display-file/file ; Reabertura do Edital PAEP nº 06/2022 - formato, pdf, 112kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24032022_Edital_1661092_Edital_6.2022_reabertura.pdf/@@display-file/file</t>
+          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4652,22 +4648,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 11/2023 - formato, pdf, 264kb</t>
+          <t>Edital PAEP nº 06/2022 - formato, pdf, 331kb</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20042023_Edital_1959492_SEI_CAPES___1959158___Edital_11_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02022022_Edital_1626836_SEI_CAPES___1626182___Edita_6.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Alteração doEdital PAEP nº 11/2023 - formato, pdf, 154kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08092023_EDITAL112023ALTERAO.pdf/@@display-file/file</t>
+          <t>Alteração do Edital PAEP nº 06/2022 - formato, pdf, 80kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15062022_Edital_1733665_Edital_6_2022.pdf/@@display-file/file ; Reabertura do Edital PAEP nº 06/2022 - formato, pdf, 112kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24032022_Edital_1661092_Edital_6.2022_reabertura.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4679,14 +4675,14 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 19/2025 - formato, pdf, 136kb</t>
+          <t>Edital PAEP nº 11/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12092025_Edital_2679718_SEI_2669828_Edital_19_2025.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20042023_Edital_1959492_SEI_CAPES___1959158___Edital_11_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -4694,7 +4690,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Alteração do edital PAEP nº 19/2025 - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23102025_Edital_2706985_SEI_2706736_Edital_n__19_2025___ALTERACAO.pdf/@@display-file/file</t>
+          <t>Alteração doEdital PAEP nº 11/2023 - formato, pdf, 154kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08092023_EDITAL112023ALTERAO.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4706,14 +4702,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 22/2024 - Alteração - formato, pdf, 47kb</t>
+          <t>Edital PAEP nº 19/2025 - formato, pdf, 136kb</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2473082_SEI_2472594_Edital_22_2024___ALTERACAO.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12092025_Edital_2679718_SEI_2669828_Edital_19_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F153" t="n">
@@ -4721,7 +4717,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 22/2024 - formato, pdf, 126kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10092024_Edital_2457107_SEI_2457028_Edital_22_2024.pdf/@@display-file/file</t>
+          <t>Alteração do edital PAEP nº 19/2025 - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23102025_Edital_2706985_SEI_2706736_Edital_n__19_2025___ALTERACAO.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4733,20 +4729,24 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 37/2023 - formato, pdf, 264kb</t>
+          <t>Edital PAEP nº 22/2024 - Alteração - formato, pdf, 47kb</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122023_Edital_2295422_SEI_2295394_Edital_37_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2473082_SEI_2472594_Edital_22_2024___ALTERACAO.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F154" t="n">
-        <v>1</v>
-      </c>
-      <c r="G154" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Edital PAEP nº 22/2024 - formato, pdf, 126kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10092024_Edital_2457107_SEI_2457028_Edital_22_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4756,24 +4756,20 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Edital PDSE nº 17/2025 – segunda chamada – relação de aprovadas na análise técnica após a análise dos recursos - formato, pdf, 1,438kb</t>
+          <t>Edital PAEP nº 37/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2878471_listagem_resultado_final_pdse_segunda_chamada.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122023_Edital_2295422_SEI_2295394_Edital_37_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F155" t="n">
-        <v>5</v>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4783,22 +4779,22 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital PDSE nº 17/2025 – segunda chamada – relação de aprovadas na análise técnica após a análise dos recursos - formato, pdf, 1,438kb</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2878471_listagem_resultado_final_pdse_segunda_chamada.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F156" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4810,20 +4806,24 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>1</v>
-      </c>
-      <c r="G157" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4833,14 +4833,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -4856,24 +4856,20 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F159" t="n">
-        <v>4</v>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -4883,14 +4879,14 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -4898,7 +4894,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4910,14 +4906,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
+          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -4925,7 +4921,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4937,22 +4933,22 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
+          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F162" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4964,37 +4960,41 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
+          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F163" t="n">
-        <v>1</v>
-      </c>
-      <c r="G163" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
+          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -5033,14 +5033,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -5056,14 +5056,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -5079,14 +5079,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -5102,14 +5102,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -5125,14 +5125,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -5148,14 +5148,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -5171,14 +5171,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -5194,14 +5194,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -5217,14 +5217,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -5240,14 +5240,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -5263,14 +5263,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -5286,14 +5286,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5309,14 +5309,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5332,14 +5332,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5355,14 +5355,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5378,14 +5378,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -5401,14 +5401,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5424,14 +5424,14 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -5447,14 +5447,14 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -5470,14 +5470,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5493,14 +5493,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5516,14 +5516,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5539,14 +5539,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5562,14 +5562,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5585,14 +5585,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -5608,24 +5608,20 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F191" t="n">
-        <v>2</v>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -5635,20 +5631,24 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
-        <v>1</v>
-      </c>
-      <c r="G192" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -5658,14 +5658,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5681,14 +5681,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5704,14 +5704,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5727,14 +5727,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -5750,14 +5750,14 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -5773,14 +5773,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5796,14 +5796,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -5819,14 +5819,14 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -5842,14 +5842,14 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -5865,14 +5865,14 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -5888,14 +5888,14 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -5911,14 +5911,14 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -5934,14 +5934,14 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F205" t="n">
@@ -5957,14 +5957,14 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F206" t="n">
@@ -5980,14 +5980,14 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F207" t="n">
@@ -6003,14 +6003,14 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F208" t="n">
@@ -6026,14 +6026,14 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr"/>
       <c r="E209" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -6049,14 +6049,14 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr"/>
       <c r="E210" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -6072,14 +6072,14 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr"/>
       <c r="E211" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -6095,24 +6095,20 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr"/>
       <c r="E212" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
         </is>
       </c>
       <c r="F212" t="n">
-        <v>2</v>
-      </c>
-      <c r="G212" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -6122,20 +6118,24 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr"/>
       <c r="E213" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
         </is>
       </c>
       <c r="F213" t="n">
-        <v>1</v>
-      </c>
-      <c r="G213" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -6145,14 +6145,14 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr"/>
       <c r="E214" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -6168,20 +6168,43 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
         </is>
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>1</v>
+      </c>
+      <c r="G215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr"/>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F215" t="n">
-        <v>1</v>
-      </c>
-      <c r="G215" t="inlineStr"/>
+      <c r="F216" t="n">
+        <v>1</v>
+      </c>
+      <c r="G216" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-09-15 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -4170,9 +4170,13 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>1</v>
-      </c>
-      <c r="G132" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Alteração Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 69,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2894158_sei_2893573_edital_n__21_2026.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">

</xml_diff>

<commit_message>
chore: crawl 2026-09-16 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -4355,9 +4355,13 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>1</v>
-      </c>
-      <c r="G139" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Alteração - Edital nº 25/2026 - Edição 2027, formato, pdf, 50,3kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2896676_sei_2896323_edital_25_2026___alteracao.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">

</xml_diff>

<commit_message>
chore: crawl 2026-09-29 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -3886,9 +3886,13 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>1</v>
-      </c>
-      <c r="G120" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2904194_sei_2903303_edital_conjunto_26_2026.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">

</xml_diff>

<commit_message>
chore: crawl 2026-10-02 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G223"/>
+  <dimension ref="A1:G227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3875,14 +3875,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Edital n° 26/2026 - Programas CAPES/MATH/STIC/CLIMAT-AMSUD, formato - pdf, 237kb</t>
+          <t>Edital n° 13/2023 - Programa de Apoio a Eventos no País para a Educação Básica (PAEP-EB) - formato, pdf, 262kb</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2891614_sei_2891436_edital_26_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24052023_Edital_1982772_SEI_CAPES___1981022___Edital_13.2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2904194_sei_2903303_edital_conjunto_26_2026.pdf/@@display-file/file</t>
+          <t>Alteração do edital n° 13/2023 - Programa de Apoio a Eventos no País para a Educação Básica (PAEP-EB) - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/27072023_Edital_2025391_Edital_13_2023_Alteracao_site.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3902,24 +3902,20 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 87kb</t>
+          <t>Edital n° 14/2024 - Programa de Apoio a Eventos no País para a Educação Básica (PAEP-EB) - formato, pdf, 102kb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/26022024_Edital_2328837_SEI_2326326_Edital_02_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14062024_Edital_2396954_SEI_2395820_Edital_14_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>2</v>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16052024_Edital_2379426_SEI_2379169_Edital_02_2024.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3929,20 +3925,24 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
+          <t>Edital n° 26/2026 - Programas CAPES/MATH/STIC/CLIMAT-AMSUD, formato - pdf, 237kb</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2891614_sei_2891436_edital_26_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>1</v>
-      </c>
-      <c r="G122" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2904194_sei_2903303_edital_conjunto_26_2026.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3952,22 +3952,22 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 87kb</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/26022024_Edital_2328837_SEI_2326326_Edital_02_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16052024_Edital_2379426_SEI_2379169_Edital_02_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3979,24 +3979,20 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
+          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>4</v>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4006,14 +4002,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -4021,7 +4017,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4029,22 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4060,14 +4056,14 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
+          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -4075,7 +4071,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4087,14 +4083,14 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
+          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -4102,7 +4098,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4114,22 +4110,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
+          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4141,20 +4137,24 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
-      </c>
-      <c r="G130" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4164,20 +4164,24 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Edital nº 14/2025 - PCI - pdf, 83kb</t>
+          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31072025_Edital_2646654_SEI_2644987_Edital_14_2025.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1</v>
-      </c>
-      <c r="G131" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4187,24 +4191,20 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
+          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F132" t="n">
-        <v>2</v>
-      </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4214,14 +4214,14 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
+          <t>Edital nº 14/2025 - PCI - pdf, 83kb</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31072025_Edital_2646654_SEI_2644987_Edital_14_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F133" t="n">
@@ -4237,20 +4237,24 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
+          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1</v>
-      </c>
-      <c r="G134" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4260,24 +4264,20 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
+          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>2</v>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>Edital nº 19/2026 - Lista de inscritos - Programa CAPES/Universidade em Buffalo (CAPES/UB) - Professor Visitante - formato, pdf, 66,7kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2892345_lista_de_inscritos.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4287,24 +4287,20 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
+          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>3</v>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4314,22 +4310,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 281kb</t>
+          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24082023_Edital_2043434_Edital_21_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Retificação do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/01112023_Edital_2262651_SEI_2262236_Edital_21_2023.pdf/@@display-file/file ; Alteração do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31102023_Edital_2261925_SEI_2261451_Edital_22_2023.pdf/@@display-file/file</t>
+          <t>Edital nº 19/2026 - Lista de inscritos - Programa CAPES/Universidade em Buffalo (CAPES/UB) - Professor Visitante - formato, pdf, 66,7kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2892345_lista_de_inscritos.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4341,22 +4337,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
+          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 69,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2894158_sei_2893573_edital_n__21_2026.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4368,22 +4364,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
+          <t>Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 281kb</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24082023_Edital_2043434_Edital_21_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Retificação do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/01112023_Edital_2262651_SEI_2262236_Edital_21_2023.pdf/@@display-file/file ; Alteração do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31102023_Edital_2261925_SEI_2261451_Edital_22_2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4395,22 +4391,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
+          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file ; Relação dos Programas de Pós-Graduação (PPGs) - Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 1.836kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/resultado_2881142_pdai_divulgacao_ppgs_bolsas_v-final_13-08-2026.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 69,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2894158_sei_2893573_edital_n__21_2026.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4422,14 +4418,14 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
+          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -4437,7 +4433,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4449,20 +4445,24 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Edital nº 24/2026 - Cooperação entre Instituições para</t>
+          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878169_edital_24_2026___pci.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1</v>
-      </c>
-      <c r="G142" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file ; Relação dos Programas de Pós-Graduação (PPGs) - Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 1.836kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/resultado_2881142_pdai_divulgacao_ppgs_bolsas_v-final_13-08-2026.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4472,22 +4472,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
+          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4499,24 +4499,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 83kb</t>
+          <t>Edital nº 24/2026 - Cooperação entre Instituições para</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/17092024_Edital_2461148_SEI_2460992_Edital_25_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878169_edital_24_2026___pci.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F144" t="n">
-        <v>2</v>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10122024_Edital_2510251_SEI_2508924_Edital_25_2024___Alteracao.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4526,22 +4522,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Edital nº 25/2026 - Edição 2027, formato, pdf, 145kb</t>
+          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2886643_sei_2886062_edital_n___25_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Alteração - Edital nº 25/2026 - Edição 2027, formato, pdf, 50,3kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2896676_sei_2896323_edital_25_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4553,22 +4549,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
+          <t>Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 83kb</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/17092024_Edital_2461148_SEI_2460992_Edital_25_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F146" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10122024_Edital_2510251_SEI_2508924_Edital_25_2024___Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4580,14 +4576,14 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
+          <t>Edital nº 25/2026 - Edição 2027, formato, pdf, 145kb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2886643_sei_2886062_edital_n___25_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F147" t="n">
@@ -4595,7 +4591,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+          <t>Alteração - Edital nº 25/2026 - Edição 2027, formato, pdf, 50,3kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2896676_sei_2896323_edital_25_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4607,14 +4603,14 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
+          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -4622,7 +4618,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4634,22 +4630,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
+          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F149" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
+          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4661,14 +4657,14 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
+          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F150" t="n">
@@ -4676,7 +4672,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4688,22 +4684,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
+          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4715,20 +4711,24 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
+          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F152" t="n">
-        <v>1</v>
-      </c>
-      <c r="G152" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4738,20 +4738,24 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
+          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F153" t="n">
-        <v>1</v>
-      </c>
-      <c r="G153" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4761,24 +4765,20 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
+          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F154" t="n">
-        <v>3</v>
-      </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4788,24 +4788,20 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F155" t="n">
-        <v>2</v>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4815,20 +4811,24 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
+          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F156" t="n">
-        <v>1</v>
-      </c>
-      <c r="G156" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
+          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4865,24 +4865,20 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 06/2022 - formato, pdf, 331kb</t>
+          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02022022_Edital_1626836_SEI_CAPES___1626182___Edita_6.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F158" t="n">
-        <v>3</v>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Alteração do Edital PAEP nº 06/2022 - formato, pdf, 80kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15062022_Edital_1733665_Edital_6_2022.pdf/@@display-file/file ; Reabertura do Edital PAEP nº 06/2022 - formato, pdf, 112kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24032022_Edital_1661092_Edital_6.2022_reabertura.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -4892,14 +4888,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 11/2023 - formato, pdf, 264kb</t>
+          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20042023_Edital_1959492_SEI_CAPES___1959158___Edital_11_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -4907,7 +4903,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Alteração doEdital PAEP nº 11/2023 - formato, pdf, 154kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08092023_EDITAL112023ALTERAO.pdf/@@display-file/file</t>
+          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4919,22 +4915,22 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 19/2025 - formato, pdf, 136kb</t>
+          <t>Edital PAEP nº 06/2022 - formato, pdf, 331kb</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12092025_Edital_2679718_SEI_2669828_Edital_19_2025.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02022022_Edital_1626836_SEI_CAPES___1626182___Edita_6.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Alteração do edital PAEP nº 19/2025 - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23102025_Edital_2706985_SEI_2706736_Edital_n__19_2025___ALTERACAO.pdf/@@display-file/file</t>
+          <t>Alteração do Edital PAEP nº 06/2022 - formato, pdf, 80kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15062022_Edital_1733665_Edital_6_2022.pdf/@@display-file/file ; Reabertura do Edital PAEP nº 06/2022 - formato, pdf, 112kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24032022_Edital_1661092_Edital_6.2022_reabertura.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4946,14 +4942,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 22/2024 - Alteração - formato, pdf, 47kb</t>
+          <t>Edital PAEP nº 11/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2473082_SEI_2472594_Edital_22_2024___ALTERACAO.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20042023_Edital_1959492_SEI_CAPES___1959158___Edital_11_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -4961,7 +4957,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 22/2024 - formato, pdf, 126kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10092024_Edital_2457107_SEI_2457028_Edital_22_2024.pdf/@@display-file/file</t>
+          <t>Alteração doEdital PAEP nº 11/2023 - formato, pdf, 154kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08092023_EDITAL112023ALTERAO.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4973,20 +4969,24 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Edital PAEP nº 37/2023 - formato, pdf, 264kb</t>
+          <t>Edital PAEP nº 19/2025 - formato, pdf, 136kb</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122023_Edital_2295422_SEI_2295394_Edital_37_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12092025_Edital_2679718_SEI_2669828_Edital_19_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F162" t="n">
-        <v>1</v>
-      </c>
-      <c r="G162" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Alteração do edital PAEP nº 19/2025 - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23102025_Edital_2706985_SEI_2706736_Edital_n__19_2025___ALTERACAO.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4996,22 +4996,22 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Edital PDSE nº 17/2025 – segunda chamada – relação de aprovadas na análise técnica após a análise dos recursos - formato, pdf, 1,438kb</t>
+          <t>Edital PAEP nº 22/2024 - Alteração - formato, pdf, 47kb</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2878471_listagem_resultado_final_pdse_segunda_chamada.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2473082_SEI_2472594_Edital_22_2024___ALTERACAO.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F163" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+          <t>Edital PAEP nº 22/2024 - formato, pdf, 126kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10092024_Edital_2457107_SEI_2457028_Edital_22_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -5023,24 +5023,20 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital PAEP nº 37/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122023_Edital_2295422_SEI_2295394_Edital_37_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F164" t="n">
-        <v>2</v>
-      </c>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5050,14 +5046,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Edital PAEP-EB nº 27/2026 - formato, pdf, 160kb</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2905712_sei_2905378_edital_27_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -5073,20 +5069,24 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Edital PDSE nº 17/2025 – segunda chamada – relação de aprovadas na análise técnica após a análise dos recursos - formato, pdf, 1,438kb</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2878471_listagem_resultado_final_pdse_segunda_chamada.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F166" t="n">
-        <v>1</v>
-      </c>
-      <c r="G166" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5096,22 +5096,22 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F167" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -5123,24 +5123,20 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F168" t="n">
-        <v>4</v>
-      </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5150,24 +5146,20 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F169" t="n">
-        <v>4</v>
-      </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5177,22 +5169,22 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F170" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -5204,106 +5196,122 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
+          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F171" t="n">
-        <v>1</v>
-      </c>
-      <c r="G171" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
+          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F172" t="n">
-        <v>1</v>
-      </c>
-      <c r="G172" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
+          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F173" t="n">
-        <v>1</v>
-      </c>
-      <c r="G173" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Prorrogação do edital n° 15/2025 - Programa de Apoio a Eventos no País para a Educação Básica (PAEP-EB) - formato, pdf, 52kb</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02102025_Edital_2693356_SEI_2692240_Edital_15_2025___Prorrogacao.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F174" t="n">
-        <v>1</v>
-      </c>
-      <c r="G174" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Prorrogação do edital PAEP-EB nº 15/2025 - formato, pdf, 575kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112025_EDITAL152025PRORROGAO.pdf/@@display-file/file ; Alteração do edital PAEP-EB nº 15/2025 - formato, pdf, 51,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13082025_Edital_2656357_SEI_2655350_Edital_15_2025.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -5319,14 +5327,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -5342,14 +5350,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5365,14 +5373,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5388,14 +5396,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5411,14 +5419,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5434,14 +5442,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -5457,14 +5465,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5480,14 +5488,14 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -5503,14 +5511,14 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -5526,14 +5534,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5549,14 +5557,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5572,14 +5580,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5595,14 +5603,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5618,14 +5626,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5641,14 +5649,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -5664,14 +5672,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -5687,14 +5695,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -5710,14 +5718,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5733,14 +5741,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5756,14 +5764,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5779,14 +5787,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -5802,14 +5810,14 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -5825,14 +5833,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5848,24 +5856,20 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F199" t="n">
-        <v>2</v>
-      </c>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -5875,14 +5879,14 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -5898,14 +5902,14 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -5921,14 +5925,14 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -5944,20 +5948,24 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F203" t="n">
-        <v>1</v>
-      </c>
-      <c r="G203" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -5967,14 +5975,14 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -5990,14 +5998,14 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F205" t="n">
@@ -6013,14 +6021,14 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F206" t="n">
@@ -6036,14 +6044,14 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F207" t="n">
@@ -6059,14 +6067,14 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F208" t="n">
@@ -6082,14 +6090,14 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr"/>
       <c r="E209" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -6105,14 +6113,14 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr"/>
       <c r="E210" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -6128,14 +6136,14 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr"/>
       <c r="E211" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -6151,14 +6159,14 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr"/>
       <c r="E212" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -6174,14 +6182,14 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr"/>
       <c r="E213" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -6197,14 +6205,14 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr"/>
       <c r="E214" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -6220,14 +6228,14 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F215" t="n">
@@ -6243,14 +6251,14 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr"/>
       <c r="E216" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F216" t="n">
@@ -6266,14 +6274,14 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F217" t="n">
@@ -6289,14 +6297,14 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr"/>
       <c r="E218" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F218" t="n">
@@ -6312,14 +6320,14 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr"/>
       <c r="E219" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F219" t="n">
@@ -6335,24 +6343,20 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr"/>
       <c r="E220" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F220" t="n">
-        <v>2</v>
-      </c>
-      <c r="G220" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -6362,14 +6366,14 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr"/>
       <c r="E221" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
         </is>
       </c>
       <c r="F221" t="n">
@@ -6385,14 +6389,14 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr"/>
       <c r="E222" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
         </is>
       </c>
       <c r="F222" t="n">
@@ -6408,20 +6412,116 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
         </is>
       </c>
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr"/>
       <c r="E223" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>1</v>
+      </c>
+      <c r="G223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr"/>
+      <c r="D224" t="inlineStr"/>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>2</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr"/>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>1</v>
+      </c>
+      <c r="G225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr"/>
+      <c r="D226" t="inlineStr"/>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>1</v>
+      </c>
+      <c r="G226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr"/>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F223" t="n">
-        <v>1</v>
-      </c>
-      <c r="G223" t="inlineStr"/>
+      <c r="F227" t="n">
+        <v>1</v>
+      </c>
+      <c r="G227" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-10-06 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -3936,11 +3936,11 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2904194_sei_2903303_edital_conjunto_26_2026.pdf/@@display-file/file</t>
+          <t>Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2904194_sei_2903303_edital_conjunto_26_2026.pdf/@@display-file/file ; Estudo de Ingressantes das Licenciaturas - Edital CAPES/INEP nº 26/2026 - Alteração | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2906989_sei_2906818_edital_conjunto_n__26_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: crawl 2026-10-16 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -1920,11 +1920,11 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Edital nº 26/2025 - Alteração, formato, pdf, 114kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878184_edital_26_2025___alteracao.pdf/@@display-file/file ; Retificação_Edital nº 26/2025 - Alteração, formato, pdf, 115kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2879083_edital_26_2025___retificacao.pdf/@@display-file/file ; Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
+          <t>Edital nº 26/2025 - Alteração, formato, pdf, 114kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878184_edital_26_2025___alteracao.pdf/@@display-file/file ; Retificação_Edital nº 26/2025 - Alteração, formato, pdf, 115kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2879083_edital_26_2025___retificacao.pdf/@@display-file/file ; Alteração - Edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato, pdf, 58,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2912764_sei_2912235_edital_26_2025___alteracao.pdf/@@display-file/file ; Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>